<commit_message>
coloacion de nueva informacion verificar por que no aumenta la informacion
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y116"/>
+  <dimension ref="A1:Y128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8266,6 +8266,810 @@
         <v>7</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2024-12-19 21:16:20</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr"/>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="n">
+        <v>10</v>
+      </c>
+      <c r="O117" t="n">
+        <v>7</v>
+      </c>
+      <c r="P117" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="n">
+        <v>1</v>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="n">
+        <v>50</v>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2024-12-19 23:44:31</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="n">
+        <v>2</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="n">
+        <v>10</v>
+      </c>
+      <c r="O118" t="n">
+        <v>7</v>
+      </c>
+      <c r="P118" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="n">
+        <v>1</v>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="n">
+        <v>15</v>
+      </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y118" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2024-12-19 23:54:42</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="n">
+        <v>14</v>
+      </c>
+      <c r="D119" t="n">
+        <v>3</v>
+      </c>
+      <c r="E119" t="n">
+        <v>5</v>
+      </c>
+      <c r="F119" t="n">
+        <v>6</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="n">
+        <v>10</v>
+      </c>
+      <c r="O119" t="n">
+        <v>7</v>
+      </c>
+      <c r="P119" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="n">
+        <v>1</v>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="n">
+        <v>50</v>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y119" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2024-12-20 21:48:51</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="n">
+        <v>12</v>
+      </c>
+      <c r="D120" t="n">
+        <v>4</v>
+      </c>
+      <c r="E120" t="n">
+        <v>7</v>
+      </c>
+      <c r="F120" t="n">
+        <v>1</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="n">
+        <v>10</v>
+      </c>
+      <c r="O120" t="n">
+        <v>7</v>
+      </c>
+      <c r="P120" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="n">
+        <v>1</v>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="n">
+        <v>50</v>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y120" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2024-12-20 22:53:48</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="n">
+        <v>17</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" t="n">
+        <v>7</v>
+      </c>
+      <c r="F121" t="n">
+        <v>9</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="n">
+        <v>10</v>
+      </c>
+      <c r="O121" t="n">
+        <v>7</v>
+      </c>
+      <c r="P121" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="n">
+        <v>1</v>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="n">
+        <v>50</v>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>39%</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr"/>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y121" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2024-12-21 00:43:49</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1</v>
+      </c>
+      <c r="E122" t="n">
+        <v>4</v>
+      </c>
+      <c r="F122" t="n">
+        <v>3</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="n">
+        <v>10</v>
+      </c>
+      <c r="O122" t="n">
+        <v>7</v>
+      </c>
+      <c r="P122" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="n">
+        <v>1</v>
+      </c>
+      <c r="S122" t="inlineStr"/>
+      <c r="T122" t="n">
+        <v>50</v>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr"/>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y122" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2024-12-21 01:01:11</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="n">
+        <v>12</v>
+      </c>
+      <c r="D123" t="n">
+        <v>4</v>
+      </c>
+      <c r="E123" t="n">
+        <v>5</v>
+      </c>
+      <c r="F123" t="n">
+        <v>3</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="n">
+        <v>10</v>
+      </c>
+      <c r="O123" t="n">
+        <v>7</v>
+      </c>
+      <c r="P123" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="n">
+        <v>1</v>
+      </c>
+      <c r="S123" t="inlineStr"/>
+      <c r="T123" t="n">
+        <v>50</v>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>71%</t>
+        </is>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr"/>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y123" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2024-12-21 01:13:54</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="n">
+        <v>9</v>
+      </c>
+      <c r="D124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E124" t="n">
+        <v>5</v>
+      </c>
+      <c r="F124" t="n">
+        <v>3</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="n">
+        <v>10</v>
+      </c>
+      <c r="O124" t="n">
+        <v>7</v>
+      </c>
+      <c r="P124" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="n">
+        <v>1</v>
+      </c>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="n">
+        <v>50</v>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr"/>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y124" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2024-12-21 01:33:36</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="n">
+        <v>6</v>
+      </c>
+      <c r="D125" t="n">
+        <v>2</v>
+      </c>
+      <c r="E125" t="n">
+        <v>2</v>
+      </c>
+      <c r="F125" t="n">
+        <v>2</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="n">
+        <v>10</v>
+      </c>
+      <c r="O125" t="n">
+        <v>7</v>
+      </c>
+      <c r="P125" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="n">
+        <v>1</v>
+      </c>
+      <c r="S125" t="inlineStr"/>
+      <c r="T125" t="n">
+        <v>50</v>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr"/>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y125" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2024-12-21 19:03:49</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="n">
+        <v>12</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>6</v>
+      </c>
+      <c r="F126" t="n">
+        <v>6</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="n">
+        <v>10</v>
+      </c>
+      <c r="O126" t="n">
+        <v>7</v>
+      </c>
+      <c r="P126" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="n">
+        <v>1</v>
+      </c>
+      <c r="S126" t="inlineStr"/>
+      <c r="T126" t="n">
+        <v>50</v>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr"/>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y126" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2024-12-21 19:21:20</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>2</v>
+      </c>
+      <c r="F127" t="n">
+        <v>4</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="n">
+        <v>10</v>
+      </c>
+      <c r="O127" t="n">
+        <v>7</v>
+      </c>
+      <c r="P127" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="n">
+        <v>1</v>
+      </c>
+      <c r="S127" t="inlineStr"/>
+      <c r="T127" t="n">
+        <v>90</v>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr"/>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y127" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2024-12-26 07:00:30</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="n">
+        <v>2</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" t="n">
+        <v>2</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="n">
+        <v>10</v>
+      </c>
+      <c r="O128" t="n">
+        <v>7</v>
+      </c>
+      <c r="P128" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="n">
+        <v>1</v>
+      </c>
+      <c r="S128" t="inlineStr"/>
+      <c r="T128" t="n">
+        <v>50</v>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr"/>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y128" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cambiar 'limite_juego' a 'limite_tardancia' en Parametro_Juego y actualizar referencias en Simulador y Main
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y128"/>
+  <dimension ref="A1:Y129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9070,6 +9070,73 @@
         <v>5</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2024-12-28 09:39:29</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="n">
+        <v>10</v>
+      </c>
+      <c r="O129" t="n">
+        <v>7</v>
+      </c>
+      <c r="P129" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="n">
+        <v>1</v>
+      </c>
+      <c r="S129" t="inlineStr"/>
+      <c r="T129" t="n">
+        <v>50</v>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr"/>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y129" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
actualizar límite de tardancia en Reporte y Main, y ajustar verificación de probabilidad en Predictor
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y129"/>
+  <dimension ref="A1:Z152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,42 +516,47 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Limite_tardancia</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Limite_pretendiente</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Probabilidad</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Efectividad</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Ruleta</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Ganancia</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Juego</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Predecidos</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Limite_juego</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Limite_pretendiente</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Probabilidad</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Efectividad</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Ruleta</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Ganancia</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Juego</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Predecidos</t>
         </is>
       </c>
     </row>
@@ -635,6 +640,7 @@
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -716,6 +722,7 @@
         </is>
       </c>
       <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -797,6 +804,7 @@
         </is>
       </c>
       <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -862,6 +870,7 @@
       <c r="Y5" t="n">
         <v>9</v>
       </c>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -927,6 +936,7 @@
       <c r="Y6" t="n">
         <v>0</v>
       </c>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -992,6 +1002,7 @@
       <c r="Y7" t="n">
         <v>5</v>
       </c>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1057,6 +1068,7 @@
       <c r="Y8" t="n">
         <v>0</v>
       </c>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1122,6 +1134,7 @@
       <c r="Y9" t="n">
         <v>3</v>
       </c>
+      <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1187,6 +1200,7 @@
       <c r="Y10" t="n">
         <v>0</v>
       </c>
+      <c r="Z10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1252,6 +1266,7 @@
       <c r="Y11" t="n">
         <v>45</v>
       </c>
+      <c r="Z11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1317,6 +1332,7 @@
       <c r="Y12" t="n">
         <v>8</v>
       </c>
+      <c r="Z12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1382,6 +1398,7 @@
       <c r="Y13" t="n">
         <v>70</v>
       </c>
+      <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1447,6 +1464,7 @@
       <c r="Y14" t="n">
         <v>97</v>
       </c>
+      <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1512,6 +1530,7 @@
       <c r="Y15" t="n">
         <v>86</v>
       </c>
+      <c r="Z15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1577,6 +1596,7 @@
       <c r="Y16" t="n">
         <v>29</v>
       </c>
+      <c r="Z16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1642,6 +1662,7 @@
       <c r="Y17" t="n">
         <v>56</v>
       </c>
+      <c r="Z17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1707,6 +1728,7 @@
       <c r="Y18" t="n">
         <v>0</v>
       </c>
+      <c r="Z18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1772,6 +1794,7 @@
       <c r="Y19" t="n">
         <v>7</v>
       </c>
+      <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1837,6 +1860,7 @@
       <c r="Y20" t="n">
         <v>0</v>
       </c>
+      <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1902,6 +1926,7 @@
       <c r="Y21" t="n">
         <v>0</v>
       </c>
+      <c r="Z21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1967,6 +1992,7 @@
       <c r="Y22" t="n">
         <v>0</v>
       </c>
+      <c r="Z22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2034,6 +2060,7 @@
       <c r="Y23" t="n">
         <v>39</v>
       </c>
+      <c r="Z23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2101,6 +2128,7 @@
       <c r="Y24" t="n">
         <v>24</v>
       </c>
+      <c r="Z24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2168,6 +2196,7 @@
       <c r="Y25" t="n">
         <v>6</v>
       </c>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2235,6 +2264,7 @@
       <c r="Y26" t="n">
         <v>29</v>
       </c>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2302,6 +2332,7 @@
       <c r="Y27" t="n">
         <v>29</v>
       </c>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2369,6 +2400,7 @@
       <c r="Y28" t="n">
         <v>98</v>
       </c>
+      <c r="Z28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2436,6 +2468,7 @@
       <c r="Y29" t="n">
         <v>34</v>
       </c>
+      <c r="Z29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2503,6 +2536,7 @@
       <c r="Y30" t="n">
         <v>0</v>
       </c>
+      <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2570,6 +2604,7 @@
       <c r="Y31" t="n">
         <v>22</v>
       </c>
+      <c r="Z31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2637,6 +2672,7 @@
       <c r="Y32" t="n">
         <v>28</v>
       </c>
+      <c r="Z32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2704,6 +2740,7 @@
       <c r="Y33" t="n">
         <v>11</v>
       </c>
+      <c r="Z33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2771,6 +2808,7 @@
       <c r="Y34" t="n">
         <v>21</v>
       </c>
+      <c r="Z34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2838,6 +2876,7 @@
       <c r="Y35" t="n">
         <v>0</v>
       </c>
+      <c r="Z35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2905,6 +2944,7 @@
       <c r="Y36" t="n">
         <v>31</v>
       </c>
+      <c r="Z36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2972,6 +3012,7 @@
       <c r="Y37" t="n">
         <v>4</v>
       </c>
+      <c r="Z37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3039,6 +3080,7 @@
       <c r="Y38" t="n">
         <v>57</v>
       </c>
+      <c r="Z38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3106,6 +3148,7 @@
       <c r="Y39" t="n">
         <v>44</v>
       </c>
+      <c r="Z39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3173,6 +3216,7 @@
       <c r="Y40" t="n">
         <v>0</v>
       </c>
+      <c r="Z40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3240,6 +3284,7 @@
       <c r="Y41" t="n">
         <v>50</v>
       </c>
+      <c r="Z41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3307,6 +3352,7 @@
       <c r="Y42" t="n">
         <v>15</v>
       </c>
+      <c r="Z42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3374,6 +3420,7 @@
       <c r="Y43" t="n">
         <v>38</v>
       </c>
+      <c r="Z43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3441,6 +3488,7 @@
       <c r="Y44" t="n">
         <v>22</v>
       </c>
+      <c r="Z44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3508,6 +3556,7 @@
       <c r="Y45" t="n">
         <v>0</v>
       </c>
+      <c r="Z45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3575,6 +3624,7 @@
       <c r="Y46" t="n">
         <v>3</v>
       </c>
+      <c r="Z46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3642,6 +3692,7 @@
       <c r="Y47" t="n">
         <v>0</v>
       </c>
+      <c r="Z47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3709,6 +3760,7 @@
       <c r="Y48" t="n">
         <v>1</v>
       </c>
+      <c r="Z48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3776,6 +3828,7 @@
       <c r="Y49" t="n">
         <v>32</v>
       </c>
+      <c r="Z49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3843,6 +3896,7 @@
       <c r="Y50" t="n">
         <v>2</v>
       </c>
+      <c r="Z50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3910,6 +3964,7 @@
       <c r="Y51" t="n">
         <v>0</v>
       </c>
+      <c r="Z51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3977,6 +4032,7 @@
       <c r="Y52" t="n">
         <v>0</v>
       </c>
+      <c r="Z52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4044,6 +4100,7 @@
       <c r="Y53" t="n">
         <v>86</v>
       </c>
+      <c r="Z53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4111,6 +4168,7 @@
       <c r="Y54" t="n">
         <v>0</v>
       </c>
+      <c r="Z54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4178,6 +4236,7 @@
       <c r="Y55" t="n">
         <v>22</v>
       </c>
+      <c r="Z55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4245,6 +4304,7 @@
       <c r="Y56" t="n">
         <v>0</v>
       </c>
+      <c r="Z56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4312,6 +4372,7 @@
       <c r="Y57" t="n">
         <v>23</v>
       </c>
+      <c r="Z57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4379,6 +4440,7 @@
       <c r="Y58" t="n">
         <v>19</v>
       </c>
+      <c r="Z58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4446,6 +4508,7 @@
       <c r="Y59" t="n">
         <v>0</v>
       </c>
+      <c r="Z59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4513,6 +4576,7 @@
       <c r="Y60" t="n">
         <v>4</v>
       </c>
+      <c r="Z60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4580,6 +4644,7 @@
       <c r="Y61" t="n">
         <v>1</v>
       </c>
+      <c r="Z61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4647,6 +4712,7 @@
       <c r="Y62" t="n">
         <v>20</v>
       </c>
+      <c r="Z62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4714,6 +4780,7 @@
       <c r="Y63" t="n">
         <v>12</v>
       </c>
+      <c r="Z63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4781,6 +4848,7 @@
       <c r="Y64" t="n">
         <v>27</v>
       </c>
+      <c r="Z64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4848,6 +4916,7 @@
       <c r="Y65" t="n">
         <v>50</v>
       </c>
+      <c r="Z65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4915,6 +4984,7 @@
       <c r="Y66" t="n">
         <v>7</v>
       </c>
+      <c r="Z66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4982,6 +5052,7 @@
       <c r="Y67" t="n">
         <v>1</v>
       </c>
+      <c r="Z67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5049,6 +5120,7 @@
       <c r="Y68" t="n">
         <v>24</v>
       </c>
+      <c r="Z68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5116,6 +5188,7 @@
       <c r="Y69" t="n">
         <v>74</v>
       </c>
+      <c r="Z69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5183,6 +5256,7 @@
       <c r="Y70" t="n">
         <v>30</v>
       </c>
+      <c r="Z70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5250,6 +5324,7 @@
       <c r="Y71" t="n">
         <v>23</v>
       </c>
+      <c r="Z71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5317,6 +5392,7 @@
       <c r="Y72" t="n">
         <v>0</v>
       </c>
+      <c r="Z72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5384,6 +5460,7 @@
       <c r="Y73" t="n">
         <v>99</v>
       </c>
+      <c r="Z73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5451,6 +5528,7 @@
       <c r="Y74" t="n">
         <v>0</v>
       </c>
+      <c r="Z74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5518,6 +5596,7 @@
       <c r="Y75" t="n">
         <v>16</v>
       </c>
+      <c r="Z75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5585,6 +5664,7 @@
       <c r="Y76" t="n">
         <v>45</v>
       </c>
+      <c r="Z76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5652,6 +5732,7 @@
       <c r="Y77" t="n">
         <v>0</v>
       </c>
+      <c r="Z77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5719,6 +5800,7 @@
       <c r="Y78" t="n">
         <v>8</v>
       </c>
+      <c r="Z78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5786,6 +5868,7 @@
       <c r="Y79" t="n">
         <v>0</v>
       </c>
+      <c r="Z79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5853,6 +5936,7 @@
       <c r="Y80" t="n">
         <v>19</v>
       </c>
+      <c r="Z80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5920,6 +6004,7 @@
       <c r="Y81" t="n">
         <v>24</v>
       </c>
+      <c r="Z81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5987,6 +6072,7 @@
       <c r="Y82" t="n">
         <v>78</v>
       </c>
+      <c r="Z82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6054,6 +6140,7 @@
       <c r="Y83" t="n">
         <v>0</v>
       </c>
+      <c r="Z83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6121,6 +6208,7 @@
       <c r="Y84" t="n">
         <v>23</v>
       </c>
+      <c r="Z84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6188,6 +6276,7 @@
       <c r="Y85" t="n">
         <v>27</v>
       </c>
+      <c r="Z85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6255,6 +6344,7 @@
       <c r="Y86" t="n">
         <v>31</v>
       </c>
+      <c r="Z86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6322,6 +6412,7 @@
       <c r="Y87" t="n">
         <v>20</v>
       </c>
+      <c r="Z87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6389,6 +6480,7 @@
       <c r="Y88" t="n">
         <v>27</v>
       </c>
+      <c r="Z88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6456,6 +6548,7 @@
       <c r="Y89" t="n">
         <v>10</v>
       </c>
+      <c r="Z89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6523,6 +6616,7 @@
       <c r="Y90" t="n">
         <v>8</v>
       </c>
+      <c r="Z90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6590,6 +6684,7 @@
       <c r="Y91" t="n">
         <v>31</v>
       </c>
+      <c r="Z91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6657,6 +6752,7 @@
       <c r="Y92" t="n">
         <v>0</v>
       </c>
+      <c r="Z92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6724,6 +6820,7 @@
       <c r="Y93" t="n">
         <v>0</v>
       </c>
+      <c r="Z93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6791,6 +6888,7 @@
       <c r="Y94" t="n">
         <v>44</v>
       </c>
+      <c r="Z94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6858,6 +6956,7 @@
       <c r="Y95" t="n">
         <v>0</v>
       </c>
+      <c r="Z95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6925,6 +7024,7 @@
       <c r="Y96" t="n">
         <v>51</v>
       </c>
+      <c r="Z96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6992,6 +7092,7 @@
       <c r="Y97" t="n">
         <v>30</v>
       </c>
+      <c r="Z97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7059,6 +7160,7 @@
       <c r="Y98" t="n">
         <v>0</v>
       </c>
+      <c r="Z98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7126,6 +7228,7 @@
       <c r="Y99" t="n">
         <v>9</v>
       </c>
+      <c r="Z99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7193,6 +7296,7 @@
       <c r="Y100" t="n">
         <v>7</v>
       </c>
+      <c r="Z100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7260,6 +7364,7 @@
       <c r="Y101" t="n">
         <v>11</v>
       </c>
+      <c r="Z101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7327,6 +7432,7 @@
       <c r="Y102" t="n">
         <v>18</v>
       </c>
+      <c r="Z102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7394,6 +7500,7 @@
       <c r="Y103" t="n">
         <v>6</v>
       </c>
+      <c r="Z103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7461,6 +7568,7 @@
       <c r="Y104" t="n">
         <v>0</v>
       </c>
+      <c r="Z104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7528,6 +7636,7 @@
       <c r="Y105" t="n">
         <v>30</v>
       </c>
+      <c r="Z105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7595,6 +7704,7 @@
       <c r="Y106" t="n">
         <v>22</v>
       </c>
+      <c r="Z106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7662,6 +7772,7 @@
       <c r="Y107" t="n">
         <v>420</v>
       </c>
+      <c r="Z107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7729,6 +7840,7 @@
       <c r="Y108" t="n">
         <v>0</v>
       </c>
+      <c r="Z108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7796,6 +7908,7 @@
       <c r="Y109" t="n">
         <v>0</v>
       </c>
+      <c r="Z109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7863,6 +7976,7 @@
       <c r="Y110" t="n">
         <v>0</v>
       </c>
+      <c r="Z110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7930,6 +8044,7 @@
       <c r="Y111" t="n">
         <v>6</v>
       </c>
+      <c r="Z111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7997,6 +8112,7 @@
       <c r="Y112" t="n">
         <v>94</v>
       </c>
+      <c r="Z112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8064,6 +8180,7 @@
       <c r="Y113" t="n">
         <v>63</v>
       </c>
+      <c r="Z113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8131,6 +8248,7 @@
       <c r="Y114" t="n">
         <v>322</v>
       </c>
+      <c r="Z114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8198,6 +8316,7 @@
       <c r="Y115" t="n">
         <v>11</v>
       </c>
+      <c r="Z115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8265,6 +8384,7 @@
       <c r="Y116" t="n">
         <v>7</v>
       </c>
+      <c r="Z116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8332,6 +8452,7 @@
       <c r="Y117" t="n">
         <v>0</v>
       </c>
+      <c r="Z117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8399,6 +8520,7 @@
       <c r="Y118" t="n">
         <v>5</v>
       </c>
+      <c r="Z118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8466,6 +8588,7 @@
       <c r="Y119" t="n">
         <v>25</v>
       </c>
+      <c r="Z119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8533,6 +8656,7 @@
       <c r="Y120" t="n">
         <v>19</v>
       </c>
+      <c r="Z120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8600,6 +8724,7 @@
       <c r="Y121" t="n">
         <v>44</v>
       </c>
+      <c r="Z121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8667,6 +8792,7 @@
       <c r="Y122" t="n">
         <v>11</v>
       </c>
+      <c r="Z122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8734,6 +8860,7 @@
       <c r="Y123" t="n">
         <v>17</v>
       </c>
+      <c r="Z123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8801,6 +8928,7 @@
       <c r="Y124" t="n">
         <v>14</v>
       </c>
+      <c r="Z124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8868,6 +8996,7 @@
       <c r="Y125" t="n">
         <v>11</v>
       </c>
+      <c r="Z125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8935,6 +9064,7 @@
       <c r="Y126" t="n">
         <v>23</v>
       </c>
+      <c r="Z126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9002,6 +9132,7 @@
       <c r="Y127" t="n">
         <v>15</v>
       </c>
+      <c r="Z127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9069,6 +9200,7 @@
       <c r="Y128" t="n">
         <v>5</v>
       </c>
+      <c r="Z128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9136,6 +9268,1571 @@
       <c r="Y129" t="n">
         <v>0</v>
       </c>
+      <c r="Z129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:04:48</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="n">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="n">
+        <v>10</v>
+      </c>
+      <c r="O130" t="n">
+        <v>7</v>
+      </c>
+      <c r="P130" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+      <c r="T130" t="n">
+        <v>50</v>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr"/>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y130" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:06:07</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="n">
+        <v>10</v>
+      </c>
+      <c r="O131" t="n">
+        <v>7</v>
+      </c>
+      <c r="P131" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr"/>
+      <c r="T131" t="n">
+        <v>50</v>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W131" t="inlineStr"/>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y131" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z131" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:09:41</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="n">
+        <v>2</v>
+      </c>
+      <c r="D132" t="n">
+        <v>2</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="n">
+        <v>10</v>
+      </c>
+      <c r="O132" t="n">
+        <v>7</v>
+      </c>
+      <c r="P132" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q132" t="inlineStr"/>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr"/>
+      <c r="T132" t="n">
+        <v>50</v>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W132" t="inlineStr"/>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y132" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z132" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:10:22</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="n">
+        <v>2</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>2</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="n">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="n">
+        <v>10</v>
+      </c>
+      <c r="O133" t="n">
+        <v>7</v>
+      </c>
+      <c r="P133" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="inlineStr"/>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+      <c r="T133" t="n">
+        <v>50</v>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr"/>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y133" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z133" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:12:10</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="n">
+        <v>2</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>2</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="n">
+        <v>10</v>
+      </c>
+      <c r="O134" t="n">
+        <v>7</v>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q134" t="inlineStr"/>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+      <c r="T134" t="n">
+        <v>50</v>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W134" t="inlineStr"/>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y134" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z134" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:13:00</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="n">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="n">
+        <v>10</v>
+      </c>
+      <c r="O135" t="n">
+        <v>7</v>
+      </c>
+      <c r="P135" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q135" t="inlineStr"/>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+      <c r="T135" t="n">
+        <v>50</v>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W135" t="inlineStr"/>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y135" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z135" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:13:12</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr"/>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="n">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="n">
+        <v>10</v>
+      </c>
+      <c r="O136" t="n">
+        <v>7</v>
+      </c>
+      <c r="P136" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+      <c r="T136" t="n">
+        <v>50</v>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr"/>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y136" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z136" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:17:05</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="n">
+        <v>18</v>
+      </c>
+      <c r="D137" t="n">
+        <v>5</v>
+      </c>
+      <c r="E137" t="n">
+        <v>13</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="n">
+        <v>10</v>
+      </c>
+      <c r="O137" t="n">
+        <v>7</v>
+      </c>
+      <c r="P137" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
+      <c r="T137" t="n">
+        <v>50</v>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr"/>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y137" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z137" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2024-12-28 10:18:25</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="n">
+        <v>5</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" t="n">
+        <v>4</v>
+      </c>
+      <c r="F138" t="n">
+        <v>1</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="n">
+        <v>10</v>
+      </c>
+      <c r="O138" t="n">
+        <v>7</v>
+      </c>
+      <c r="P138" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr"/>
+      <c r="T138" t="n">
+        <v>50</v>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr"/>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y138" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z138" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2024-12-28 11:41:17</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" t="n">
+        <v>3</v>
+      </c>
+      <c r="F139" t="n">
+        <v>1</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="n">
+        <v>10</v>
+      </c>
+      <c r="O139" t="n">
+        <v>7</v>
+      </c>
+      <c r="P139" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="n">
+        <v>1</v>
+      </c>
+      <c r="S139" t="inlineStr"/>
+      <c r="T139" t="n">
+        <v>20</v>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y139" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2024-12-28 11:43:14</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="n">
+        <v>7</v>
+      </c>
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" t="n">
+        <v>4</v>
+      </c>
+      <c r="F140" t="n">
+        <v>2</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="n">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="n">
+        <v>10</v>
+      </c>
+      <c r="O140" t="n">
+        <v>7</v>
+      </c>
+      <c r="P140" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="n">
+        <v>1</v>
+      </c>
+      <c r="S140" t="inlineStr"/>
+      <c r="T140" t="n">
+        <v>20</v>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W140" t="inlineStr"/>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y140" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2024-12-28 18:25:42</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="n">
+        <v>10</v>
+      </c>
+      <c r="O141" t="n">
+        <v>7</v>
+      </c>
+      <c r="P141" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="n">
+        <v>5</v>
+      </c>
+      <c r="S141" t="inlineStr"/>
+      <c r="T141" t="n">
+        <v>70</v>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y141" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2024-12-28 18:27:04</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="n">
+        <v>10</v>
+      </c>
+      <c r="O142" t="n">
+        <v>7</v>
+      </c>
+      <c r="P142" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="n">
+        <v>5</v>
+      </c>
+      <c r="S142" t="inlineStr"/>
+      <c r="T142" t="n">
+        <v>70</v>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr"/>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y142" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2024-12-28 18:29:02</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="n">
+        <v>10</v>
+      </c>
+      <c r="O143" t="n">
+        <v>7</v>
+      </c>
+      <c r="P143" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="n">
+        <v>5</v>
+      </c>
+      <c r="S143" t="inlineStr"/>
+      <c r="T143" t="n">
+        <v>70</v>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W143" t="inlineStr"/>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y143" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2024-12-28 18:31:28</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="n">
+        <v>3</v>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" t="n">
+        <v>1</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="n">
+        <v>10</v>
+      </c>
+      <c r="O144" t="n">
+        <v>7</v>
+      </c>
+      <c r="P144" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="n">
+        <v>5</v>
+      </c>
+      <c r="S144" t="inlineStr"/>
+      <c r="T144" t="n">
+        <v>70</v>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr"/>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y144" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2024-12-28 18:34:55</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="n">
+        <v>14</v>
+      </c>
+      <c r="D145" t="n">
+        <v>3</v>
+      </c>
+      <c r="E145" t="n">
+        <v>6</v>
+      </c>
+      <c r="F145" t="n">
+        <v>5</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="n">
+        <v>10</v>
+      </c>
+      <c r="O145" t="n">
+        <v>7</v>
+      </c>
+      <c r="P145" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="n">
+        <v>10</v>
+      </c>
+      <c r="S145" t="inlineStr"/>
+      <c r="T145" t="n">
+        <v>70</v>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W145" t="inlineStr"/>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y145" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2024-12-28 21:58:49</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="n">
+        <v>7</v>
+      </c>
+      <c r="D146" t="n">
+        <v>3</v>
+      </c>
+      <c r="E146" t="n">
+        <v>1</v>
+      </c>
+      <c r="F146" t="n">
+        <v>3</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="n">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="n">
+        <v>10</v>
+      </c>
+      <c r="O146" t="n">
+        <v>7</v>
+      </c>
+      <c r="P146" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="n">
+        <v>10</v>
+      </c>
+      <c r="S146" t="inlineStr"/>
+      <c r="T146" t="n">
+        <v>90</v>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr"/>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y146" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:08:18</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="n">
+        <v>24</v>
+      </c>
+      <c r="D147" t="n">
+        <v>8</v>
+      </c>
+      <c r="E147" t="n">
+        <v>10</v>
+      </c>
+      <c r="F147" t="n">
+        <v>6</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="n">
+        <v>10</v>
+      </c>
+      <c r="O147" t="n">
+        <v>7</v>
+      </c>
+      <c r="P147" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="n">
+        <v>5</v>
+      </c>
+      <c r="S147" t="inlineStr"/>
+      <c r="T147" t="n">
+        <v>50</v>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y147" t="n">
+        <v>69</v>
+      </c>
+      <c r="Z147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:17:35</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="n">
+        <v>7</v>
+      </c>
+      <c r="D148" t="n">
+        <v>2</v>
+      </c>
+      <c r="E148" t="n">
+        <v>3</v>
+      </c>
+      <c r="F148" t="n">
+        <v>2</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="n">
+        <v>10</v>
+      </c>
+      <c r="O148" t="n">
+        <v>7</v>
+      </c>
+      <c r="P148" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q148" t="inlineStr"/>
+      <c r="R148" t="n">
+        <v>5</v>
+      </c>
+      <c r="S148" t="inlineStr"/>
+      <c r="T148" t="n">
+        <v>50</v>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr"/>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y148" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:18:22</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="n">
+        <v>2</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" t="n">
+        <v>1</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="n">
+        <v>10</v>
+      </c>
+      <c r="O149" t="n">
+        <v>7</v>
+      </c>
+      <c r="P149" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="n">
+        <v>5</v>
+      </c>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="n">
+        <v>1</v>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y149" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:18:31</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr"/>
+      <c r="N150" t="n">
+        <v>10</v>
+      </c>
+      <c r="O150" t="n">
+        <v>7</v>
+      </c>
+      <c r="P150" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="n">
+        <v>5</v>
+      </c>
+      <c r="S150" t="inlineStr"/>
+      <c r="T150" t="n">
+        <v>1</v>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr"/>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y150" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:18:42</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr"/>
+      <c r="N151" t="n">
+        <v>10</v>
+      </c>
+      <c r="O151" t="n">
+        <v>7</v>
+      </c>
+      <c r="P151" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="n">
+        <v>1</v>
+      </c>
+      <c r="S151" t="inlineStr"/>
+      <c r="T151" t="n">
+        <v>1</v>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr"/>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y151" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2024-12-30 00:20:54</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr"/>
+      <c r="C152" t="n">
+        <v>11</v>
+      </c>
+      <c r="D152" t="n">
+        <v>11</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr"/>
+      <c r="N152" t="n">
+        <v>10</v>
+      </c>
+      <c r="O152" t="n">
+        <v>7</v>
+      </c>
+      <c r="P152" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q152" t="inlineStr"/>
+      <c r="R152" t="n">
+        <v>3</v>
+      </c>
+      <c r="S152" t="inlineStr"/>
+      <c r="T152" t="n">
+        <v>1</v>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y152" t="n">
+        <v>337</v>
+      </c>
+      <c r="Z152" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
se jugaron partidas en crupier
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z152"/>
+  <dimension ref="A1:Z158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10834,6 +10834,414 @@
       </c>
       <c r="Z152" t="inlineStr"/>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2025-01-01 23:50:34</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="n">
+        <v>9</v>
+      </c>
+      <c r="D153" t="n">
+        <v>5</v>
+      </c>
+      <c r="E153" t="n">
+        <v>3</v>
+      </c>
+      <c r="F153" t="n">
+        <v>1</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="n">
+        <v>10</v>
+      </c>
+      <c r="O153" t="n">
+        <v>7</v>
+      </c>
+      <c r="P153" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="n">
+        <v>5</v>
+      </c>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="n">
+        <v>90</v>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y153" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2025-01-01 23:51:32</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr"/>
+      <c r="N154" t="n">
+        <v>10</v>
+      </c>
+      <c r="O154" t="n">
+        <v>7</v>
+      </c>
+      <c r="P154" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="n">
+        <v>5</v>
+      </c>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="n">
+        <v>90</v>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y154" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2025-01-01 23:52:40</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="n">
+        <v>0</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="n">
+        <v>10</v>
+      </c>
+      <c r="O155" t="n">
+        <v>7</v>
+      </c>
+      <c r="P155" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="n">
+        <v>5</v>
+      </c>
+      <c r="S155" t="inlineStr"/>
+      <c r="T155" t="n">
+        <v>90</v>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y155" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2025-01-02 00:01:52</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>1</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr"/>
+      <c r="N156" t="n">
+        <v>10</v>
+      </c>
+      <c r="O156" t="n">
+        <v>7</v>
+      </c>
+      <c r="P156" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="n">
+        <v>5</v>
+      </c>
+      <c r="S156" t="inlineStr"/>
+      <c r="T156" t="n">
+        <v>90</v>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W156" t="inlineStr"/>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y156" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2025-01-02 00:05:35</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="n">
+        <v>4</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="n">
+        <v>2</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr"/>
+      <c r="N157" t="n">
+        <v>10</v>
+      </c>
+      <c r="O157" t="n">
+        <v>7</v>
+      </c>
+      <c r="P157" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="n">
+        <v>5</v>
+      </c>
+      <c r="S157" t="inlineStr"/>
+      <c r="T157" t="n">
+        <v>90</v>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr"/>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y157" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2025-01-02 00:16:38</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" t="n">
+        <v>1</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr"/>
+      <c r="N158" t="n">
+        <v>10</v>
+      </c>
+      <c r="O158" t="n">
+        <v>7</v>
+      </c>
+      <c r="P158" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="n">
+        <v>5</v>
+      </c>
+      <c r="S158" t="inlineStr"/>
+      <c r="T158" t="n">
+        <v>90</v>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr"/>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y158" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z158" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert "se jugaron partidas en crupier"
This reverts commit fcff1fdea6831fc6fa3776588e465a280a499409.
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z158"/>
+  <dimension ref="A1:Z152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10834,414 +10834,6 @@
       </c>
       <c r="Z152" t="inlineStr"/>
     </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>2025-01-01 23:50:34</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="n">
-        <v>9</v>
-      </c>
-      <c r="D153" t="n">
-        <v>5</v>
-      </c>
-      <c r="E153" t="n">
-        <v>3</v>
-      </c>
-      <c r="F153" t="n">
-        <v>1</v>
-      </c>
-      <c r="G153" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" t="n">
-        <v>0</v>
-      </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
-      <c r="M153" t="inlineStr"/>
-      <c r="N153" t="n">
-        <v>10</v>
-      </c>
-      <c r="O153" t="n">
-        <v>7</v>
-      </c>
-      <c r="P153" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q153" t="inlineStr"/>
-      <c r="R153" t="n">
-        <v>5</v>
-      </c>
-      <c r="S153" t="inlineStr"/>
-      <c r="T153" t="n">
-        <v>90</v>
-      </c>
-      <c r="U153" t="inlineStr">
-        <is>
-          <t>43%</t>
-        </is>
-      </c>
-      <c r="V153" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
-        </is>
-      </c>
-      <c r="W153" t="inlineStr"/>
-      <c r="X153" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y153" t="n">
-        <v>21</v>
-      </c>
-      <c r="Z153" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>2025-01-01 23:51:32</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="n">
-        <v>0</v>
-      </c>
-      <c r="D154" t="n">
-        <v>0</v>
-      </c>
-      <c r="E154" t="n">
-        <v>0</v>
-      </c>
-      <c r="F154" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" t="n">
-        <v>0</v>
-      </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
-      <c r="N154" t="n">
-        <v>10</v>
-      </c>
-      <c r="O154" t="n">
-        <v>7</v>
-      </c>
-      <c r="P154" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q154" t="inlineStr"/>
-      <c r="R154" t="n">
-        <v>5</v>
-      </c>
-      <c r="S154" t="inlineStr"/>
-      <c r="T154" t="n">
-        <v>90</v>
-      </c>
-      <c r="U154" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V154" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
-        </is>
-      </c>
-      <c r="W154" t="inlineStr"/>
-      <c r="X154" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y154" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z154" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>2025-01-01 23:52:40</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr"/>
-      <c r="C155" t="n">
-        <v>0</v>
-      </c>
-      <c r="D155" t="n">
-        <v>0</v>
-      </c>
-      <c r="E155" t="n">
-        <v>0</v>
-      </c>
-      <c r="F155" t="n">
-        <v>0</v>
-      </c>
-      <c r="G155" t="n">
-        <v>0</v>
-      </c>
-      <c r="H155" t="n">
-        <v>0</v>
-      </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
-      <c r="M155" t="inlineStr"/>
-      <c r="N155" t="n">
-        <v>10</v>
-      </c>
-      <c r="O155" t="n">
-        <v>7</v>
-      </c>
-      <c r="P155" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q155" t="inlineStr"/>
-      <c r="R155" t="n">
-        <v>5</v>
-      </c>
-      <c r="S155" t="inlineStr"/>
-      <c r="T155" t="n">
-        <v>90</v>
-      </c>
-      <c r="U155" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V155" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
-        </is>
-      </c>
-      <c r="W155" t="inlineStr"/>
-      <c r="X155" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y155" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z155" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>2025-01-02 00:01:52</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="n">
-        <v>1</v>
-      </c>
-      <c r="D156" t="n">
-        <v>0</v>
-      </c>
-      <c r="E156" t="n">
-        <v>1</v>
-      </c>
-      <c r="F156" t="n">
-        <v>0</v>
-      </c>
-      <c r="G156" t="n">
-        <v>0</v>
-      </c>
-      <c r="H156" t="n">
-        <v>0</v>
-      </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
-      <c r="M156" t="inlineStr"/>
-      <c r="N156" t="n">
-        <v>10</v>
-      </c>
-      <c r="O156" t="n">
-        <v>7</v>
-      </c>
-      <c r="P156" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="n">
-        <v>5</v>
-      </c>
-      <c r="S156" t="inlineStr"/>
-      <c r="T156" t="n">
-        <v>90</v>
-      </c>
-      <c r="U156" t="inlineStr">
-        <is>
-          <t>12%</t>
-        </is>
-      </c>
-      <c r="V156" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
-        </is>
-      </c>
-      <c r="W156" t="inlineStr"/>
-      <c r="X156" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y156" t="n">
-        <v>8</v>
-      </c>
-      <c r="Z156" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>2025-01-02 00:05:35</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="n">
-        <v>4</v>
-      </c>
-      <c r="D157" t="n">
-        <v>1</v>
-      </c>
-      <c r="E157" t="n">
-        <v>2</v>
-      </c>
-      <c r="F157" t="n">
-        <v>1</v>
-      </c>
-      <c r="G157" t="n">
-        <v>0</v>
-      </c>
-      <c r="H157" t="n">
-        <v>0</v>
-      </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
-      <c r="M157" t="inlineStr"/>
-      <c r="N157" t="n">
-        <v>10</v>
-      </c>
-      <c r="O157" t="n">
-        <v>7</v>
-      </c>
-      <c r="P157" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q157" t="inlineStr"/>
-      <c r="R157" t="n">
-        <v>5</v>
-      </c>
-      <c r="S157" t="inlineStr"/>
-      <c r="T157" t="n">
-        <v>90</v>
-      </c>
-      <c r="U157" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="V157" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
-        </is>
-      </c>
-      <c r="W157" t="inlineStr"/>
-      <c r="X157" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y157" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z157" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>2025-01-02 00:16:38</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr"/>
-      <c r="C158" t="n">
-        <v>2</v>
-      </c>
-      <c r="D158" t="n">
-        <v>1</v>
-      </c>
-      <c r="E158" t="n">
-        <v>0</v>
-      </c>
-      <c r="F158" t="n">
-        <v>1</v>
-      </c>
-      <c r="G158" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I158" t="inlineStr"/>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
-      <c r="M158" t="inlineStr"/>
-      <c r="N158" t="n">
-        <v>10</v>
-      </c>
-      <c r="O158" t="n">
-        <v>7</v>
-      </c>
-      <c r="P158" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q158" t="inlineStr"/>
-      <c r="R158" t="n">
-        <v>5</v>
-      </c>
-      <c r="S158" t="inlineStr"/>
-      <c r="T158" t="n">
-        <v>90</v>
-      </c>
-      <c r="U158" t="inlineStr">
-        <is>
-          <t>33%</t>
-        </is>
-      </c>
-      <c r="V158" t="inlineStr">
-        <is>
-          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
-        </is>
-      </c>
-      <c r="W158" t="inlineStr"/>
-      <c r="X158" t="inlineStr">
-        <is>
-          <t>No es Simulación</t>
-        </is>
-      </c>
-      <c r="Y158" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z158" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar cálculo de frecuencia y normalización en el modelo de predicción
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z152"/>
+  <dimension ref="A1:Z156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10834,6 +10834,278 @@
       </c>
       <c r="Z152" t="inlineStr"/>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2025-01-03 00:19:49</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="n">
+        <v>10</v>
+      </c>
+      <c r="O153" t="n">
+        <v>7</v>
+      </c>
+      <c r="P153" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="n">
+        <v>5</v>
+      </c>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="n">
+        <v>50</v>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y153" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2025-01-03 00:25:32</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="n">
+        <v>9</v>
+      </c>
+      <c r="D154" t="n">
+        <v>2</v>
+      </c>
+      <c r="E154" t="n">
+        <v>4</v>
+      </c>
+      <c r="F154" t="n">
+        <v>3</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr"/>
+      <c r="N154" t="n">
+        <v>10</v>
+      </c>
+      <c r="O154" t="n">
+        <v>7</v>
+      </c>
+      <c r="P154" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="n">
+        <v>5</v>
+      </c>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="n">
+        <v>50</v>
+      </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>41%</t>
+        </is>
+      </c>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y154" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2025-01-03 00:32:28</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="n">
+        <v>14</v>
+      </c>
+      <c r="D155" t="n">
+        <v>4</v>
+      </c>
+      <c r="E155" t="n">
+        <v>6</v>
+      </c>
+      <c r="F155" t="n">
+        <v>4</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="n">
+        <v>10</v>
+      </c>
+      <c r="O155" t="n">
+        <v>7</v>
+      </c>
+      <c r="P155" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="n">
+        <v>5</v>
+      </c>
+      <c r="S155" t="inlineStr"/>
+      <c r="T155" t="n">
+        <v>50</v>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>37%</t>
+        </is>
+      </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y155" t="n">
+        <v>38</v>
+      </c>
+      <c r="Z155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2025-01-03 00:34:23</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr"/>
+      <c r="N156" t="n">
+        <v>10</v>
+      </c>
+      <c r="O156" t="n">
+        <v>7</v>
+      </c>
+      <c r="P156" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="n">
+        <v>5</v>
+      </c>
+      <c r="S156" t="inlineStr"/>
+      <c r="T156" t="n">
+        <v>10</v>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W156" t="inlineStr"/>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y156" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z156" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar sectores en el modelo de predicción y ajustar filtrado de predicciones; implementar decorador para modificar tardanza en la clase NumeroJugar.
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z156"/>
+  <dimension ref="A1:Z161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11106,6 +11106,346 @@
       </c>
       <c r="Z156" t="inlineStr"/>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2025-01-04 14:30:17</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="n">
+        <v>3</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" t="n">
+        <v>1</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr"/>
+      <c r="N157" t="n">
+        <v>10</v>
+      </c>
+      <c r="O157" t="n">
+        <v>7</v>
+      </c>
+      <c r="P157" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="n">
+        <v>5</v>
+      </c>
+      <c r="S157" t="inlineStr"/>
+      <c r="T157" t="n">
+        <v>50</v>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>19%</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr"/>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y157" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2025-01-05 07:21:19</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="n">
+        <v>5</v>
+      </c>
+      <c r="D158" t="n">
+        <v>2</v>
+      </c>
+      <c r="E158" t="n">
+        <v>3</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr"/>
+      <c r="N158" t="n">
+        <v>10</v>
+      </c>
+      <c r="O158" t="n">
+        <v>7</v>
+      </c>
+      <c r="P158" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="n">
+        <v>2</v>
+      </c>
+      <c r="S158" t="inlineStr"/>
+      <c r="T158" t="n">
+        <v>50</v>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr"/>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y158" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2025-01-05 07:22:04</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr"/>
+      <c r="C159" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="inlineStr"/>
+      <c r="N159" t="n">
+        <v>10</v>
+      </c>
+      <c r="O159" t="n">
+        <v>7</v>
+      </c>
+      <c r="P159" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q159" t="inlineStr"/>
+      <c r="R159" t="n">
+        <v>2</v>
+      </c>
+      <c r="S159" t="inlineStr"/>
+      <c r="T159" t="n">
+        <v>90</v>
+      </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V159" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W159" t="inlineStr"/>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y159" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2025-01-05 07:28:40</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr"/>
+      <c r="C160" t="n">
+        <v>3</v>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" t="n">
+        <v>2</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr"/>
+      <c r="N160" t="n">
+        <v>10</v>
+      </c>
+      <c r="O160" t="n">
+        <v>7</v>
+      </c>
+      <c r="P160" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q160" t="inlineStr"/>
+      <c r="R160" t="n">
+        <v>2</v>
+      </c>
+      <c r="S160" t="inlineStr"/>
+      <c r="T160" t="n">
+        <v>90</v>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr"/>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y160" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2025-01-05 07:34:26</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr"/>
+      <c r="C161" t="n">
+        <v>17</v>
+      </c>
+      <c r="D161" t="n">
+        <v>17</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="inlineStr"/>
+      <c r="N161" t="n">
+        <v>10</v>
+      </c>
+      <c r="O161" t="n">
+        <v>7</v>
+      </c>
+      <c r="P161" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q161" t="inlineStr"/>
+      <c r="R161" t="n">
+        <v>2</v>
+      </c>
+      <c r="S161" t="inlineStr"/>
+      <c r="T161" t="n">
+        <v>10</v>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W161" t="inlineStr"/>
+      <c r="X161" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y161" t="n">
+        <v>114</v>
+      </c>
+      <c r="Z161" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Eliminar código comentado y características innecesarias en las clases NumeroJugar y Modelo
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z161"/>
+  <dimension ref="A1:Z163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11446,6 +11446,142 @@
       </c>
       <c r="Z161" t="inlineStr"/>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2025-01-06 03:16:16</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="n">
+        <v>10</v>
+      </c>
+      <c r="O162" t="n">
+        <v>7</v>
+      </c>
+      <c r="P162" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" t="inlineStr"/>
+      <c r="T162" t="n">
+        <v>50</v>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr"/>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y162" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2025-01-06 03:21:13</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr"/>
+      <c r="C163" t="n">
+        <v>5</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" t="n">
+        <v>2</v>
+      </c>
+      <c r="F163" t="n">
+        <v>2</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="n">
+        <v>1</v>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="inlineStr"/>
+      <c r="N163" t="n">
+        <v>10</v>
+      </c>
+      <c r="O163" t="n">
+        <v>7</v>
+      </c>
+      <c r="P163" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q163" t="inlineStr"/>
+      <c r="R163" t="n">
+        <v>5</v>
+      </c>
+      <c r="S163" t="inlineStr"/>
+      <c r="T163" t="n">
+        <v>50</v>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W163" t="inlineStr"/>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y163" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z163" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Eliminar la columna 'vecinos2' y ajustar el tamaño de entrada en la capa de embedding del modelo de predicción
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z161"/>
+  <dimension ref="A1:Z162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11446,6 +11446,74 @@
       </c>
       <c r="Z161" t="inlineStr"/>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2025-01-08 18:34:00</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="n">
+        <v>5</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" t="n">
+        <v>3</v>
+      </c>
+      <c r="F162" t="n">
+        <v>1</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="n">
+        <v>10</v>
+      </c>
+      <c r="O162" t="n">
+        <v>7</v>
+      </c>
+      <c r="P162" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" t="inlineStr"/>
+      <c r="T162" t="n">
+        <v>50</v>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr"/>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y162" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z162" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar la columna 'vecino1' para utilizar datos de 'Salidos' en lugar de 'vecino2'
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z163"/>
+  <dimension ref="A1:Z170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11582,6 +11582,482 @@
       </c>
       <c r="Z163" t="inlineStr"/>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2025-01-09 02:17:59</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr"/>
+      <c r="C164" t="n">
+        <v>17</v>
+      </c>
+      <c r="D164" t="n">
+        <v>4</v>
+      </c>
+      <c r="E164" t="n">
+        <v>4</v>
+      </c>
+      <c r="F164" t="n">
+        <v>9</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr"/>
+      <c r="M164" t="inlineStr"/>
+      <c r="N164" t="n">
+        <v>10</v>
+      </c>
+      <c r="O164" t="n">
+        <v>7</v>
+      </c>
+      <c r="P164" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q164" t="inlineStr"/>
+      <c r="R164" t="n">
+        <v>5</v>
+      </c>
+      <c r="S164" t="inlineStr"/>
+      <c r="T164" t="n">
+        <v>50</v>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W164" t="inlineStr"/>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y164" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2025-01-09 02:19:16</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr"/>
+      <c r="C165" t="n">
+        <v>2</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" t="n">
+        <v>1</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
+      <c r="M165" t="inlineStr"/>
+      <c r="N165" t="n">
+        <v>10</v>
+      </c>
+      <c r="O165" t="n">
+        <v>7</v>
+      </c>
+      <c r="P165" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q165" t="inlineStr"/>
+      <c r="R165" t="n">
+        <v>5</v>
+      </c>
+      <c r="S165" t="inlineStr"/>
+      <c r="T165" t="n">
+        <v>50</v>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W165" t="inlineStr"/>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y165" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2025-01-09 02:27:32</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="n">
+        <v>12</v>
+      </c>
+      <c r="D166" t="n">
+        <v>4</v>
+      </c>
+      <c r="E166" t="n">
+        <v>6</v>
+      </c>
+      <c r="F166" t="n">
+        <v>2</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="n">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr"/>
+      <c r="M166" t="inlineStr"/>
+      <c r="N166" t="n">
+        <v>10</v>
+      </c>
+      <c r="O166" t="n">
+        <v>7</v>
+      </c>
+      <c r="P166" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q166" t="inlineStr"/>
+      <c r="R166" t="n">
+        <v>5</v>
+      </c>
+      <c r="S166" t="inlineStr"/>
+      <c r="T166" t="n">
+        <v>50</v>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>39%</t>
+        </is>
+      </c>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W166" t="inlineStr"/>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y166" t="n">
+        <v>31</v>
+      </c>
+      <c r="Z166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2025-01-10 20:36:12</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr"/>
+      <c r="C167" t="n">
+        <v>20</v>
+      </c>
+      <c r="D167" t="n">
+        <v>3</v>
+      </c>
+      <c r="E167" t="n">
+        <v>9</v>
+      </c>
+      <c r="F167" t="n">
+        <v>8</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>3</v>
+      </c>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr"/>
+      <c r="M167" t="inlineStr"/>
+      <c r="N167" t="n">
+        <v>10</v>
+      </c>
+      <c r="O167" t="n">
+        <v>7</v>
+      </c>
+      <c r="P167" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q167" t="inlineStr"/>
+      <c r="R167" t="n">
+        <v>5</v>
+      </c>
+      <c r="S167" t="inlineStr"/>
+      <c r="T167" t="n">
+        <v>50</v>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr"/>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y167" t="n">
+        <v>40</v>
+      </c>
+      <c r="Z167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2025-01-10 21:06:33</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr"/>
+      <c r="C168" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="n">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="n">
+        <v>10</v>
+      </c>
+      <c r="O168" t="n">
+        <v>7</v>
+      </c>
+      <c r="P168" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q168" t="inlineStr"/>
+      <c r="R168" t="n">
+        <v>5</v>
+      </c>
+      <c r="S168" t="inlineStr"/>
+      <c r="T168" t="n">
+        <v>50</v>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Crupier.xlsx</t>
+        </is>
+      </c>
+      <c r="W168" t="inlineStr"/>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y168" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2025-01-11 18:27:36</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr"/>
+      <c r="C169" t="n">
+        <v>34</v>
+      </c>
+      <c r="D169" t="n">
+        <v>4</v>
+      </c>
+      <c r="E169" t="n">
+        <v>15</v>
+      </c>
+      <c r="F169" t="n">
+        <v>15</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="n">
+        <v>5</v>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="n">
+        <v>10</v>
+      </c>
+      <c r="O169" t="n">
+        <v>7</v>
+      </c>
+      <c r="P169" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q169" t="inlineStr"/>
+      <c r="R169" t="n">
+        <v>5</v>
+      </c>
+      <c r="S169" t="inlineStr"/>
+      <c r="T169" t="n">
+        <v>50</v>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="V169" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W169" t="inlineStr"/>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y169" t="n">
+        <v>76</v>
+      </c>
+      <c r="Z169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2025-01-11 18:29:17</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr"/>
+      <c r="C170" t="n">
+        <v>5</v>
+      </c>
+      <c r="D170" t="n">
+        <v>1</v>
+      </c>
+      <c r="E170" t="n">
+        <v>2</v>
+      </c>
+      <c r="F170" t="n">
+        <v>2</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="n">
+        <v>10</v>
+      </c>
+      <c r="O170" t="n">
+        <v>7</v>
+      </c>
+      <c r="P170" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="n">
+        <v>5</v>
+      </c>
+      <c r="S170" t="inlineStr"/>
+      <c r="T170" t="n">
+        <v>50</v>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr"/>
+      <c r="X170" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y170" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z170" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactorizar la función de predicción para mejorar el filtrado de resultados y eliminar números con probabilidad cero.
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z161"/>
+  <dimension ref="A1:Z173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11446,6 +11446,822 @@
       </c>
       <c r="Z161" t="inlineStr"/>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2025-01-26 19:56:38</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="n">
+        <v>29</v>
+      </c>
+      <c r="D162" t="n">
+        <v>5</v>
+      </c>
+      <c r="E162" t="n">
+        <v>15</v>
+      </c>
+      <c r="F162" t="n">
+        <v>9</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="n">
+        <v>10</v>
+      </c>
+      <c r="O162" t="n">
+        <v>10</v>
+      </c>
+      <c r="P162" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" t="inlineStr"/>
+      <c r="T162" t="n">
+        <v>50</v>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr"/>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y162" t="n">
+        <v>65</v>
+      </c>
+      <c r="Z162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2025-01-27 17:56:18</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr"/>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="n">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="inlineStr"/>
+      <c r="N163" t="n">
+        <v>10</v>
+      </c>
+      <c r="O163" t="n">
+        <v>10</v>
+      </c>
+      <c r="P163" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q163" t="inlineStr"/>
+      <c r="R163" t="n">
+        <v>5</v>
+      </c>
+      <c r="S163" t="inlineStr"/>
+      <c r="T163" t="n">
+        <v>50</v>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W163" t="inlineStr"/>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y163" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2025-01-27 17:56:36</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr"/>
+      <c r="C164" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0</v>
+      </c>
+      <c r="F164" t="n">
+        <v>0</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr"/>
+      <c r="M164" t="inlineStr"/>
+      <c r="N164" t="n">
+        <v>10</v>
+      </c>
+      <c r="O164" t="n">
+        <v>10</v>
+      </c>
+      <c r="P164" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q164" t="inlineStr"/>
+      <c r="R164" t="n">
+        <v>1</v>
+      </c>
+      <c r="S164" t="inlineStr"/>
+      <c r="T164" t="n">
+        <v>50</v>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W164" t="inlineStr"/>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y164" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2025-01-27 20:16:21</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr"/>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
+      <c r="M165" t="inlineStr"/>
+      <c r="N165" t="n">
+        <v>10</v>
+      </c>
+      <c r="O165" t="n">
+        <v>10</v>
+      </c>
+      <c r="P165" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q165" t="inlineStr"/>
+      <c r="R165" t="n">
+        <v>1</v>
+      </c>
+      <c r="S165" t="inlineStr"/>
+      <c r="T165" t="n">
+        <v>20</v>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>11%</t>
+        </is>
+      </c>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W165" t="inlineStr"/>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y165" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:03:00</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0</v>
+      </c>
+      <c r="F166" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="n">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr"/>
+      <c r="M166" t="inlineStr"/>
+      <c r="N166" t="n">
+        <v>10</v>
+      </c>
+      <c r="O166" t="n">
+        <v>10</v>
+      </c>
+      <c r="P166" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q166" t="inlineStr"/>
+      <c r="R166" t="n">
+        <v>1</v>
+      </c>
+      <c r="S166" t="inlineStr"/>
+      <c r="T166" t="n">
+        <v>50</v>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W166" t="inlineStr"/>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y166" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2025-01-27 21:36:38</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr"/>
+      <c r="C167" t="n">
+        <v>4</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+      <c r="E167" t="n">
+        <v>2</v>
+      </c>
+      <c r="F167" t="n">
+        <v>2</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr"/>
+      <c r="M167" t="inlineStr"/>
+      <c r="N167" t="n">
+        <v>10</v>
+      </c>
+      <c r="O167" t="n">
+        <v>10</v>
+      </c>
+      <c r="P167" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q167" t="inlineStr"/>
+      <c r="R167" t="n">
+        <v>1</v>
+      </c>
+      <c r="S167" t="inlineStr"/>
+      <c r="T167" t="n">
+        <v>20</v>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr"/>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y167" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:20:09</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr"/>
+      <c r="C168" t="n">
+        <v>4</v>
+      </c>
+      <c r="D168" t="n">
+        <v>2</v>
+      </c>
+      <c r="E168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F168" t="n">
+        <v>1</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="n">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="n">
+        <v>10</v>
+      </c>
+      <c r="O168" t="n">
+        <v>10</v>
+      </c>
+      <c r="P168" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q168" t="inlineStr"/>
+      <c r="R168" t="n">
+        <v>3</v>
+      </c>
+      <c r="S168" t="inlineStr"/>
+      <c r="T168" t="n">
+        <v>20</v>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W168" t="inlineStr"/>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y168" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:27:59</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr"/>
+      <c r="C169" t="n">
+        <v>6</v>
+      </c>
+      <c r="D169" t="n">
+        <v>2</v>
+      </c>
+      <c r="E169" t="n">
+        <v>2</v>
+      </c>
+      <c r="F169" t="n">
+        <v>2</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="n">
+        <v>10</v>
+      </c>
+      <c r="O169" t="n">
+        <v>10</v>
+      </c>
+      <c r="P169" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q169" t="inlineStr"/>
+      <c r="R169" t="n">
+        <v>3</v>
+      </c>
+      <c r="S169" t="inlineStr"/>
+      <c r="T169" t="n">
+        <v>20</v>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="V169" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W169" t="inlineStr"/>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y169" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:30:47</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr"/>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="n">
+        <v>10</v>
+      </c>
+      <c r="O170" t="n">
+        <v>10</v>
+      </c>
+      <c r="P170" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q170" t="inlineStr"/>
+      <c r="R170" t="n">
+        <v>3</v>
+      </c>
+      <c r="S170" t="inlineStr"/>
+      <c r="T170" t="n">
+        <v>20</v>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr"/>
+      <c r="X170" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y170" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:31:23</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr"/>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="n">
+        <v>0</v>
+      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="n">
+        <v>10</v>
+      </c>
+      <c r="O171" t="n">
+        <v>10</v>
+      </c>
+      <c r="P171" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q171" t="inlineStr"/>
+      <c r="R171" t="n">
+        <v>3</v>
+      </c>
+      <c r="S171" t="inlineStr"/>
+      <c r="T171" t="n">
+        <v>20</v>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W171" t="inlineStr"/>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y171" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:46:28</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr"/>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="n">
+        <v>0</v>
+      </c>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="inlineStr"/>
+      <c r="N172" t="n">
+        <v>10</v>
+      </c>
+      <c r="O172" t="n">
+        <v>10</v>
+      </c>
+      <c r="P172" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q172" t="inlineStr"/>
+      <c r="R172" t="n">
+        <v>5</v>
+      </c>
+      <c r="S172" t="inlineStr"/>
+      <c r="T172" t="n">
+        <v>50</v>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V172" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W172" t="inlineStr"/>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y172" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2025-01-27 23:48:17</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr"/>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>0</v>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="n">
+        <v>10</v>
+      </c>
+      <c r="O173" t="n">
+        <v>10</v>
+      </c>
+      <c r="P173" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q173" t="inlineStr"/>
+      <c r="R173" t="n">
+        <v>5</v>
+      </c>
+      <c r="S173" t="inlineStr"/>
+      <c r="T173" t="n">
+        <v>40</v>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V173" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W173" t="inlineStr"/>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y173" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z173" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor imports to follow consistent naming conventions and improve code readability.
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z173"/>
+  <dimension ref="A1:Z175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12262,6 +12262,142 @@
       </c>
       <c r="Z173" t="inlineStr"/>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2025-01-29 23:02:23</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr"/>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" t="n">
+        <v>0</v>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="n">
+        <v>10</v>
+      </c>
+      <c r="O174" t="n">
+        <v>10</v>
+      </c>
+      <c r="P174" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q174" t="inlineStr"/>
+      <c r="R174" t="n">
+        <v>5</v>
+      </c>
+      <c r="S174" t="inlineStr"/>
+      <c r="T174" t="n">
+        <v>30</v>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W174" t="inlineStr"/>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y174" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2025-01-29 23:47:59</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr"/>
+      <c r="C175" t="n">
+        <v>0</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="n">
+        <v>0</v>
+      </c>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="n">
+        <v>10</v>
+      </c>
+      <c r="O175" t="n">
+        <v>10</v>
+      </c>
+      <c r="P175" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q175" t="inlineStr"/>
+      <c r="R175" t="n">
+        <v>5</v>
+      </c>
+      <c r="S175" t="inlineStr"/>
+      <c r="T175" t="n">
+        <v>50</v>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>C:\Users\jonat\OneDrive\Escritorio\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W175" t="inlineStr"/>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y175" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z175" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Increase the number of optimization trials from 30 to 100
</commit_message>
<xml_diff>
--- a/Data/Reporte_juego.xlsx
+++ b/Data/Reporte_juego.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z161"/>
+  <dimension ref="A1:Z162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11446,6 +11446,74 @@
       </c>
       <c r="Z161" t="inlineStr"/>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2025-02-05 18:27:38</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="n">
+        <v>10</v>
+      </c>
+      <c r="O162" t="n">
+        <v>10</v>
+      </c>
+      <c r="P162" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q162" t="inlineStr"/>
+      <c r="R162" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" t="inlineStr"/>
+      <c r="T162" t="n">
+        <v>50</v>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>D:\Repositorio\jonatha1992\Predictor_ruleta\Data\Electromecanica.xlsx</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr"/>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>No es Simulación</t>
+        </is>
+      </c>
+      <c r="Y162" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z162" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>